<commit_message>
Add rounded-card layout file; drop Bauhaus styling
New editable Letter-size layout (pptx) for Canva or Google Slides with
rounded cards and a faint shadow. The Sheet goes back to plain Inter and
stays the calculator and event log.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017uhWxcvQLLnDQKisxUaLUC
</commit_message>
<xml_diff>
--- a/one-pager/368-Hellhound-OnePager.xlsx
+++ b/one-pager/368-Hellhound-OnePager.xlsx
@@ -39,187 +39,187 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="00171717"/>
       <sz val="24"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <color rgb="006B6B6B"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="000096CF"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="00171717"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <color rgb="006B6B6B"/>
       <sz val="10.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <color rgb="00E8382F"/>
       <sz val="10.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <i val="1"/>
       <color rgb="006B6B6B"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="00171717"/>
       <sz val="20"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <color rgb="00171717"/>
       <sz val="10.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <color rgb="00E8382F"/>
       <sz val="9.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <color rgb="006B6B6B"/>
       <sz val="9.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="006B6B6B"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <color rgb="006B6B6B"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="00171717"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <color rgb="00171717"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="00E8382F"/>
       <sz val="10.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="006B6B6B"/>
       <sz val="8.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <color rgb="006B6B6B"/>
       <sz val="8.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="000096CF"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="00171717"/>
       <sz val="32"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <color rgb="006B6B6B"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="00171717"/>
       <sz val="15"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="00171717"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="00171717"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="00E8382F"/>
       <sz val="8.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="00A3A3A3"/>
       <sz val="8"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
-      <color rgb="00171717"/>
+      <color rgb="000096CF"/>
       <sz val="8.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="00171717"/>
       <sz val="9.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <color rgb="00171717"/>
       <sz val="9.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <color rgb="00A3A3A3"/>
       <sz val="8.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <b val="1"/>
       <color rgb="00171717"/>
       <sz val="10.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <i val="1"/>
       <color rgb="006B6B6B"/>
       <sz val="10.5"/>
     </font>
     <font>
-      <name val="Jost"/>
+      <name val="Inter"/>
       <i val="1"/>
       <color rgb="00A3A3A3"/>
       <sz val="10"/>
@@ -362,17 +362,17 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="bottom" indent="3"/>
+      <alignment horizontal="left" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="24" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" indent="3"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="2"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="25" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -403,7 +403,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="bottom" indent="2"/>
+      <alignment horizontal="left" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -615,281 +615,6 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>7</col>
-      <colOff>762000</colOff>
-      <row>3</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1714500" cy="1714500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>14</row>
-      <rowOff>85725</rowOff>
-    </from>
-    <ext cx="171450" cy="171450"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>85725</rowOff>
-    </from>
-    <ext cx="171450" cy="171450"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Image 3" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>20</row>
-      <rowOff>85725</rowOff>
-    </from>
-    <ext cx="171450" cy="171450"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="4" name="Image 4" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>23</row>
-      <rowOff>85725</rowOff>
-    </from>
-    <ext cx="171450" cy="171450"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Image 5" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>9525</colOff>
-      <row>29</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="66675" cy="66675"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="6" name="Image 6" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>9525</colOff>
-      <row>30</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="66675" cy="66675"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="7" name="Image 7" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>9525</colOff>
-      <row>31</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="66675" cy="66675"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="8" name="Image 8" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>9525</colOff>
-      <row>29</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="66675" cy="66675"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="9" name="Image 9" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>9525</colOff>
-      <row>30</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="66675" cy="66675"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="10" name="Image 10" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>9525</colOff>
-      <row>31</row>
-      <rowOff>76200</rowOff>
-    </from>
-    <ext cx="66675" cy="66675"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="11" name="Image 11" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
       <col>1</col>
       <colOff>0</colOff>
       <row>38</row>
@@ -898,11 +623,11 @@
     <ext cx="533400" cy="533400"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -923,116 +648,11 @@
     <ext cx="1638300" cy="504825"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="13" name="Image 13" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>8</row>
-      <rowOff>85725</rowOff>
-    </from>
-    <ext cx="104775" cy="104775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>11</row>
-      <rowOff>85725</rowOff>
-    </from>
-    <ext cx="104775" cy="104775"/>
-    <pic>
-      <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>15</row>
-      <rowOff>85725</rowOff>
-    </from>
-    <ext cx="104775" cy="104775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Image 3" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>85725</rowOff>
-    </from>
-    <ext cx="104775" cy="104775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="4" name="Image 4" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1588,11 +1208,8 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n"/>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Font: Jost. If it shows as Arial, pick Format › Font › More fonts › Jost once and it will load.</t>
-        </is>
-      </c>
+      <c r="B27" s="1" t="n"/>
+      <c r="C27" s="1" t="n"/>
       <c r="D27" s="1" t="n"/>
     </row>
     <row r="28">
@@ -1608,13 +1225,12 @@
       <c r="D29" s="1" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="5">
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="1" fitToWidth="1"/>
@@ -2036,7 +1652,7 @@
       <c r="A30" s="9" t="n"/>
       <c r="B30" s="22" t="inlineStr">
         <is>
-          <t>Backup computer, running live</t>
+          <t>✓  Backup computer, running live</t>
         </is>
       </c>
       <c r="C30" s="23" t="n"/>
@@ -2045,7 +1661,7 @@
       <c r="F30" s="9" t="n"/>
       <c r="G30" s="22" t="inlineStr">
         <is>
-          <t>Lead engineer on site</t>
+          <t>✓  Lead engineer on site</t>
         </is>
       </c>
       <c r="H30" s="23" t="n"/>
@@ -2057,7 +1673,7 @@
       <c r="A31" s="9" t="n"/>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>Wired internet with cellular backup</t>
+          <t>✓  Wired internet with cellular backup</t>
         </is>
       </c>
       <c r="C31" s="23" t="n"/>
@@ -2066,7 +1682,7 @@
       <c r="F31" s="9" t="n"/>
       <c r="G31" s="22" t="inlineStr">
         <is>
-          <t>Full rehearsal the day before</t>
+          <t>✓  Full rehearsal the day before</t>
         </is>
       </c>
       <c r="H31" s="23" t="n"/>
@@ -2078,7 +1694,7 @@
       <c r="A32" s="9" t="n"/>
       <c r="B32" s="22" t="inlineStr">
         <is>
-          <t>A mic for every speaker</t>
+          <t>✓  A mic for every speaker</t>
         </is>
       </c>
       <c r="C32" s="23" t="n"/>
@@ -2087,7 +1703,7 @@
       <c r="F32" s="9" t="n"/>
       <c r="G32" s="22" t="inlineStr">
         <is>
-          <t>Delivery, setup, and teardown</t>
+          <t>✓  Delivery, setup, and teardown</t>
         </is>
       </c>
       <c r="H32" s="23" t="n"/>
@@ -2938,7 +2554,6 @@
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>